<commit_message>
Fill in the estimation for P1
</commit_message>
<xml_diff>
--- a/Product_Backlog/Product_Backlog.xlsx
+++ b/Product_Backlog/Product_Backlog.xlsx
@@ -801,7 +801,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -852,13 +852,6 @@
       <color rgb="FF000000"/>
       <name val="微软雅黑"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -1384,148 +1377,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="8" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -2492,7 +2485,9 @@
       <c r="F14" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="G14" s="19"/>
+      <c r="G14" s="19">
+        <v>2</v>
+      </c>
       <c r="H14" s="20"/>
       <c r="I14" s="22"/>
       <c r="J14" s="22"/>
@@ -2516,7 +2511,9 @@
       <c r="F15" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="G15" s="14"/>
+      <c r="G15" s="14">
+        <v>2</v>
+      </c>
       <c r="H15" s="15"/>
       <c r="I15" s="18"/>
       <c r="J15" s="18"/>
@@ -2540,7 +2537,9 @@
       <c r="F16" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="G16" s="19"/>
+      <c r="G16" s="19">
+        <v>2</v>
+      </c>
       <c r="H16" s="20" t="s">
         <v>74</v>
       </c>
@@ -2566,7 +2565,9 @@
       <c r="F17" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="G17" s="14"/>
+      <c r="G17" s="14">
+        <v>1</v>
+      </c>
       <c r="H17" s="15"/>
       <c r="I17" s="18"/>
       <c r="J17" s="18"/>
@@ -2590,7 +2591,9 @@
       <c r="F18" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="G18" s="19"/>
+      <c r="G18" s="19">
+        <v>2</v>
+      </c>
       <c r="H18" s="20"/>
       <c r="I18" s="22"/>
       <c r="J18" s="22"/>
@@ -2614,7 +2617,9 @@
       <c r="F19" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="G19" s="14"/>
+      <c r="G19" s="14">
+        <v>1</v>
+      </c>
       <c r="H19" s="15"/>
       <c r="I19" s="18"/>
       <c r="J19" s="18"/>
@@ -2638,7 +2643,9 @@
       <c r="F20" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="G20" s="19"/>
+      <c r="G20" s="19">
+        <v>2</v>
+      </c>
       <c r="H20" s="20"/>
       <c r="I20" s="22"/>
       <c r="J20" s="22"/>
@@ -2662,7 +2669,9 @@
       <c r="F21" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="G21" s="14"/>
+      <c r="G21" s="14">
+        <v>2</v>
+      </c>
       <c r="H21" s="15"/>
       <c r="I21" s="18"/>
       <c r="J21" s="18"/>
@@ -2686,7 +2695,9 @@
       <c r="F22" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="G22" s="19"/>
+      <c r="G22" s="19">
+        <v>2</v>
+      </c>
       <c r="H22" s="20"/>
       <c r="I22" s="22"/>
       <c r="J22" s="22"/>
@@ -2710,7 +2721,9 @@
       <c r="F23" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="G23" s="14"/>
+      <c r="G23" s="14">
+        <v>1</v>
+      </c>
       <c r="H23" s="15"/>
       <c r="I23" s="18"/>
       <c r="J23" s="18"/>
@@ -2734,7 +2747,9 @@
       <c r="F24" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="G24" s="19"/>
+      <c r="G24" s="19">
+        <v>2</v>
+      </c>
       <c r="H24" s="20"/>
       <c r="I24" s="22"/>
       <c r="J24" s="22"/>
@@ -2758,7 +2773,9 @@
       <c r="F25" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="G25" s="14"/>
+      <c r="G25" s="14">
+        <v>2</v>
+      </c>
       <c r="H25" s="15"/>
       <c r="I25" s="18"/>
       <c r="J25" s="18"/>
@@ -2782,7 +2799,9 @@
       <c r="F26" s="21" t="s">
         <v>114</v>
       </c>
-      <c r="G26" s="19"/>
+      <c r="G26" s="19">
+        <v>1</v>
+      </c>
       <c r="H26" s="20"/>
       <c r="I26" s="22"/>
       <c r="J26" s="22"/>

</xml_diff>

<commit_message>
Fill in the estimation for P2
</commit_message>
<xml_diff>
--- a/Product_Backlog/Product_Backlog.xlsx
+++ b/Product_Backlog/Product_Backlog.xlsx
@@ -2825,7 +2825,9 @@
       <c r="F27" s="16" t="s">
         <v>119</v>
       </c>
-      <c r="G27" s="14"/>
+      <c r="G27" s="14">
+        <v>2</v>
+      </c>
       <c r="H27" s="15"/>
       <c r="I27" s="18"/>
       <c r="J27" s="18"/>
@@ -2849,7 +2851,9 @@
       <c r="F28" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="G28" s="19"/>
+      <c r="G28" s="19">
+        <v>2</v>
+      </c>
       <c r="H28" s="20" t="s">
         <v>124</v>
       </c>
@@ -2875,7 +2879,9 @@
       <c r="F29" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="G29" s="14"/>
+      <c r="G29" s="14">
+        <v>2</v>
+      </c>
       <c r="H29" s="15" t="s">
         <v>129</v>
       </c>
@@ -2901,7 +2907,9 @@
       <c r="F30" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="G30" s="19"/>
+      <c r="G30" s="19">
+        <v>2</v>
+      </c>
       <c r="H30" s="20"/>
       <c r="I30" s="22"/>
       <c r="J30" s="22"/>
@@ -2925,7 +2933,9 @@
       <c r="F31" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="G31" s="14"/>
+      <c r="G31" s="14">
+        <v>2</v>
+      </c>
       <c r="H31" s="15"/>
       <c r="I31" s="18"/>
       <c r="J31" s="18"/>
@@ -2949,7 +2959,9 @@
       <c r="F32" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="G32" s="19"/>
+      <c r="G32" s="19">
+        <v>1</v>
+      </c>
       <c r="H32" s="20"/>
       <c r="I32" s="22"/>
       <c r="J32" s="22"/>
@@ -2973,7 +2985,9 @@
       <c r="F33" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="G33" s="14"/>
+      <c r="G33" s="14">
+        <v>2</v>
+      </c>
       <c r="H33" s="15"/>
       <c r="I33" s="18"/>
       <c r="J33" s="18"/>
@@ -2997,7 +3011,9 @@
       <c r="F34" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="G34" s="19"/>
+      <c r="G34" s="19">
+        <v>2</v>
+      </c>
       <c r="H34" s="20"/>
       <c r="I34" s="22"/>
       <c r="J34" s="22"/>
@@ -3021,7 +3037,9 @@
       <c r="F35" s="16" t="s">
         <v>153</v>
       </c>
-      <c r="G35" s="14"/>
+      <c r="G35" s="14">
+        <v>1</v>
+      </c>
       <c r="H35" s="15"/>
       <c r="I35" s="18"/>
       <c r="J35" s="18"/>
@@ -3045,7 +3063,9 @@
       <c r="F36" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="G36" s="19"/>
+      <c r="G36" s="19">
+        <v>2</v>
+      </c>
       <c r="H36" s="20" t="s">
         <v>158</v>
       </c>
@@ -3071,7 +3091,9 @@
       <c r="F37" s="16" t="s">
         <v>162</v>
       </c>
-      <c r="G37" s="14"/>
+      <c r="G37" s="14">
+        <v>1</v>
+      </c>
       <c r="H37" s="15"/>
       <c r="I37" s="18"/>
       <c r="J37" s="18"/>
@@ -3095,7 +3117,9 @@
       <c r="F38" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="G38" s="19"/>
+      <c r="G38" s="19">
+        <v>2</v>
+      </c>
       <c r="H38" s="20"/>
       <c r="I38" s="22"/>
       <c r="J38" s="22"/>
@@ -3119,7 +3143,9 @@
       <c r="F39" s="16" t="s">
         <v>170</v>
       </c>
-      <c r="G39" s="14"/>
+      <c r="G39" s="14">
+        <v>2</v>
+      </c>
       <c r="H39" s="15"/>
       <c r="I39" s="18"/>
       <c r="J39" s="18"/>
@@ -3143,7 +3169,9 @@
       <c r="F40" s="21" t="s">
         <v>174</v>
       </c>
-      <c r="G40" s="19"/>
+      <c r="G40" s="19">
+        <v>1</v>
+      </c>
       <c r="H40" s="20"/>
       <c r="I40" s="22"/>
       <c r="J40" s="22"/>
@@ -3167,7 +3195,9 @@
       <c r="F41" s="16" t="s">
         <v>178</v>
       </c>
-      <c r="G41" s="14"/>
+      <c r="G41" s="14">
+        <v>2</v>
+      </c>
       <c r="H41" s="15"/>
       <c r="I41" s="18"/>
       <c r="J41" s="18"/>
@@ -3191,7 +3221,9 @@
       <c r="F42" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="G42" s="19"/>
+      <c r="G42" s="19">
+        <v>1</v>
+      </c>
       <c r="H42" s="20"/>
       <c r="I42" s="22"/>
       <c r="J42" s="22"/>

</xml_diff>

<commit_message>
Fill in the estimation for P3
</commit_message>
<xml_diff>
--- a/Product_Backlog/Product_Backlog.xlsx
+++ b/Product_Backlog/Product_Backlog.xlsx
@@ -3247,7 +3247,9 @@
       <c r="F43" s="16" t="s">
         <v>187</v>
       </c>
-      <c r="G43" s="14"/>
+      <c r="G43" s="14">
+        <v>2</v>
+      </c>
       <c r="H43" s="15" t="s">
         <v>188</v>
       </c>
@@ -3273,7 +3275,9 @@
       <c r="F44" s="21" t="s">
         <v>192</v>
       </c>
-      <c r="G44" s="19"/>
+      <c r="G44" s="19">
+        <v>1</v>
+      </c>
       <c r="H44" s="20"/>
       <c r="I44" s="22"/>
       <c r="J44" s="22"/>
@@ -3297,7 +3301,9 @@
       <c r="F45" s="16" t="s">
         <v>196</v>
       </c>
-      <c r="G45" s="14"/>
+      <c r="G45" s="14">
+        <v>1</v>
+      </c>
       <c r="H45" s="15"/>
       <c r="I45" s="18"/>
       <c r="J45" s="18"/>
@@ -3321,7 +3327,9 @@
       <c r="F46" s="21" t="s">
         <v>200</v>
       </c>
-      <c r="G46" s="19"/>
+      <c r="G46" s="19">
+        <v>2</v>
+      </c>
       <c r="H46" s="20"/>
       <c r="I46" s="22"/>
       <c r="J46" s="22"/>
@@ -3345,7 +3353,9 @@
       <c r="F47" s="16" t="s">
         <v>204</v>
       </c>
-      <c r="G47" s="14"/>
+      <c r="G47" s="14">
+        <v>1</v>
+      </c>
       <c r="H47" s="15"/>
       <c r="I47" s="18"/>
       <c r="J47" s="18"/>
@@ -3369,7 +3379,9 @@
       <c r="F48" s="21" t="s">
         <v>208</v>
       </c>
-      <c r="G48" s="19"/>
+      <c r="G48" s="19">
+        <v>2</v>
+      </c>
       <c r="H48" s="20"/>
       <c r="I48" s="22"/>
       <c r="J48" s="22"/>
@@ -3393,7 +3405,9 @@
       <c r="F49" s="16" t="s">
         <v>212</v>
       </c>
-      <c r="G49" s="14"/>
+      <c r="G49" s="14">
+        <v>2</v>
+      </c>
       <c r="H49" s="15"/>
       <c r="I49" s="18"/>
       <c r="J49" s="18"/>
@@ -3417,7 +3431,9 @@
       <c r="F50" s="21" t="s">
         <v>216</v>
       </c>
-      <c r="G50" s="19"/>
+      <c r="G50" s="19">
+        <v>1</v>
+      </c>
       <c r="H50" s="20"/>
       <c r="I50" s="22"/>
       <c r="J50" s="22"/>

</xml_diff>